<commit_message>
Latest generated outputs 2026-08-04
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/approval-of-details-reserved-by-condition-approval-condition.xlsx
+++ b/generated/spreadsheet/approval-of-details-reserved-by-condition-approval-condition.xlsx
@@ -427,17 +427,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="72" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -491,29 +491,29 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The details of the application payload to be submitted</t>
+          <t>Details about the submitted payload, including how it is identified, routed, validated, handled and traced</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Submission reference</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>A unique reference for the submission</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -532,7 +532,7 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -563,19 +563,19 @@
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Planning authority</t>
+          <t>Specification profile</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>A reference of the planning authority the application has been submitted to, e.g. local-authority:CMD for London borough of Camden</t>
+          <t>The specification profile used to determine context-specific allowed codelist values for the application</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -594,24 +594,24 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Submission date</t>
+          <t>Planning authority</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Date the application is submitted in YYYY-MM-DD format</t>
+          <t>A reference of the planning authority the application has been submitted to, e.g. local-authority:CMD for London borough of Camden</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -625,24 +625,24 @@
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Modules[]</t>
+          <t>Submitted at</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>List of required modules for this application that can be used to validate the application</t>
+          <t>The date and time the application was submitted</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -656,28 +656,24 @@
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Documents[]</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
+          <t>Created at</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Unique reference for the document within this application submission, generated by the submitting system</t>
+          <t>The date and time the submission payload was created</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -691,7 +687,7 @@
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -701,13 +697,13 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>The name or title of the document</t>
+          <t>Unique reference for the document within this application submission, generated by the submitting system</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -726,7 +722,7 @@
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -736,13 +732,13 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Brief description of what the document contains</t>
+          <t>The name or title of the document</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -752,7 +748,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -761,7 +757,7 @@
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -771,23 +767,23 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Document types[]</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>List of codelist references that the document covers</t>
+          <t>Brief description of what the document contains</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -796,7 +792,7 @@
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -806,18 +802,18 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Uploaded date</t>
+          <t>Document types[]</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>The date the document was uploaded to the application</t>
+          <t>List of codelist references that the document covers</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -831,7 +827,7 @@
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -841,27 +837,23 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Base64</t>
-        </is>
-      </c>
+          <t>Uploaded date</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Base64-encoded content of the file for inline file uploads</t>
+          <t>The date the document was uploaded to the application</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -870,7 +862,7 @@
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -885,12 +877,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Filename</t>
+          <t>Base64</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Name of the file being uploaded</t>
+          <t>Base64-encoded content of the file for inline file uploads</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -900,7 +892,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -909,7 +901,7 @@
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -924,12 +916,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>MIME type</t>
+          <t>Filename</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>The file's MIME type such as application/pdf or image/jpeg</t>
+          <t>Name of the file being uploaded</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -939,7 +931,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -948,7 +940,7 @@
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -963,17 +955,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>File size</t>
+          <t>MIME type</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Size of the file in bytes that can be used to enforce limits</t>
+          <t>The file's MIME type such as application/pdf or image/jpeg</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -987,33 +979,37 @@
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Fee</t>
+          <t>Documents[]</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>File size</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>The total amount due for the application fee</t>
+          <t>Size of the file in bytes that can be used to enforce limits</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1018,7 @@
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1032,18 +1028,18 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Amount paid</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>The amount paid towards the application fee</t>
+          <t>The total amount due for the application fee</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1057,7 +1053,7 @@
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Submission details</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1067,48 +1063,48 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Transactions[]</t>
+          <t>Amount paid</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>References to payments or financial transactions related to this application</t>
+          <t>The amount paid towards the application fee</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Agent contact details</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information if an agent is being used.</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Agent reference</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>Submission details</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Fee</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Transactions[]</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>A reference to an agent object</t>
+          <t>References to payments or financial transactions related to this application</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1118,28 +1114,32 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Agent contact details</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information if an agent is being used.</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Contact details</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
+          <t>Agent reference</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>A reference to an agent object</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1163,18 +1163,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Phone number(s)[]</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Phone number</t>
-        </is>
-      </c>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1184,7 +1180,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1203,18 +1199,18 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Contact priority</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>The priority of a number</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1224,47 +1220,51 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Agent details</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information if an agent is being used.</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>agent</t>
+          <t>Contact details</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
+          <t>Phone number(s)[]</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Contact priority</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>The priority of a number</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Agent details</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information if an agent is being used.</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>agent</t>
@@ -1272,18 +1272,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>The title of the individual</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1293,7 +1289,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1308,13 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>The first name of the individual</t>
+          <t>The title of the individual</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1328,7 +1324,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1347,13 +1343,13 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>The last name of the individual</t>
+          <t>The first name of the individual</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1382,13 +1378,13 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The last name of the individual</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1417,13 +1413,13 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1433,7 +1429,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1447,14 +1443,18 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>The name of a company (that the agent works for)</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1478,19 +1478,19 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>User role</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>The role of the named individual. Agent or proxy</t>
+          <t>The name of a company (that the agent works for)</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1500,58 +1500,58 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Applicant contact details</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Telephone number and email address of the applicant.</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Applicant reference</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>User role</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Reference to match contact details to a named individual from the applicant details component</t>
+          <t>The role of the named individual. Agent or proxy</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Applicant contact details</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Telephone number and email address of the applicant.</t>
+        </is>
+      </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Contact details</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
+          <t>Applicant reference</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>Reference to match contact details to a named individual from the applicant details component</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1575,18 +1575,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Phone number(s)[]</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Phone number</t>
-        </is>
-      </c>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1596,7 +1592,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1615,18 +1611,18 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Contact priority</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>The priority of a number</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -1636,47 +1632,51 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Applicant details</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information for the parties making the application.</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Applicants[]</t>
+          <t>Contact details</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
+          <t>Phone number(s)[]</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Contact priority</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>The priority of a number</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Applicant details</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information for the parties making the application.</t>
+        </is>
+      </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Applicants[]</t>
@@ -1684,18 +1684,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>The title of the individual</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1705,7 +1701,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1724,13 +1720,13 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>The first name of the individual</t>
+          <t>The title of the individual</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1740,7 +1736,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1759,13 +1755,13 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>The last name of the individual</t>
+          <t>The first name of the individual</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1794,13 +1790,13 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The last name of the individual</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -1829,13 +1825,13 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1845,32 +1841,32 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Checklist</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Checking whether all the requirements of the form have been met, such as proof of payment or supporting documentation.</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>National requirement types[]</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
+          <t>Applicants[]</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
       <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>List of the document types required for the given application type</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -1880,70 +1876,78 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Conflict of interest</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
+          <t>Checking whether all the requirements of the form have been met, such as proof of payment or supporting documentation.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>National requirement types[]</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>List of the document types required for the given application type</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Declaration</t>
+          <t>Conflict of interest</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Signed and dated verification of the application's accuracy.</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
+          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>A name of a person</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Declaration</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Signed and dated verification of the application's accuracy.</t>
+        </is>
+      </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Declaration confirmed</t>
+          <t>Person reference</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
@@ -1951,12 +1955,12 @@
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
+          <t>Declaration must be made by an applicant or agent making the application</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -1970,7 +1974,7 @@
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Declaration date</t>
+          <t>Declaration confirmed</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
@@ -1978,12 +1982,12 @@
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>The date the declaration was made</t>
+          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -1993,36 +1997,24 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Description of your proposal</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Written description of the proposed development including any additional relevant details.</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Related application</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
+          <t>Declaration date</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>The reference for the related application</t>
+          <t>The date the declaration was made</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2032,8 +2024,16 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Description of your proposal</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Written description of the proposed development including any additional relevant details.</t>
+        </is>
+      </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Related application</t>
@@ -2041,14 +2041,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>A description of the related application</t>
+          <t>The reference for the related application</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2072,24 +2072,24 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Decision date</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>The date when the decision was made, in YYYY-MM-DD format</t>
+          <t>A description of the related application</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2098,20 +2098,24 @@
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Condition numbers[]</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
+          <t>Related application</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Decision date</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>List of condition numbers related to this application</t>
+          <t>The date when the decision was made, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -2125,7 +2129,7 @@
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Has development started</t>
+          <t>Condition numbers[]</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
@@ -2133,17 +2137,17 @@
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Whether the development has already started</t>
+          <t>List of condition numbers related to this application</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2156,7 @@
       <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Development start date</t>
+          <t>Has development started</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
@@ -2160,17 +2164,17 @@
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Date when development started</t>
+          <t>Whether the development has already started</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2183,7 @@
       <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Has development completed</t>
+          <t>Development start date</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
@@ -2187,17 +2191,17 @@
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Whether the development has been completed</t>
+          <t>Date when development started</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2210,7 @@
       <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Development completed date</t>
+          <t>Has development completed</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -2214,34 +2218,26 @@
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Date when development was completed</t>
+          <t>Whether the development has been completed</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Discharge condition</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>How any conditions imposed as part of being given planning permission will be met</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Description list</t>
+          <t>Development completed date</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
@@ -2249,34 +2245,34 @@
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Description or list of materials/details that are being submitted for approval</t>
+          <t>Date when development was completed</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Part discharge</t>
+          <t>Discharge condition</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Details of how the applicant is meeting a specific part of a set of conditions made by the planning authority.</t>
+          <t>How any conditions imposed as part of being given planning permission will be met</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Is discharging part</t>
+          <t>Description list</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -2284,12 +2280,12 @@
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Is applicant trying to discharge part of condition?</t>
+          <t>Description or list of materials/details that are being submitted for approval</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -2299,11 +2295,19 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Part discharge</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Details of how the applicant is meeting a specific part of a set of conditions made by the planning authority.</t>
+        </is>
+      </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Discharging part details</t>
+          <t>Is discharging part</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -2311,34 +2315,26 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Indicate which part of the condition the application relates to</t>
+          <t>Is applicant trying to discharge part of condition?</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Pre-application advice</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Details of pre-application advice previously received from the planning authority</t>
-        </is>
-      </c>
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Pre-application advice sought</t>
+          <t>Discharging part details</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -2346,26 +2342,34 @@
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Whether pre-application advice has been sought from the planning authority</t>
+          <t>Indicate which part of the condition the application relates to</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Pre-application advice</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Details of pre-application advice previously received from the planning authority</t>
+        </is>
+      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Officer name</t>
+          <t>Pre-application advice sought</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -2373,17 +2377,17 @@
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Name of the planning officer who provided the pre-application advice</t>
+          <t>Whether pre-application advice has been sought from the planning authority</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2396,7 @@
       <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Officer name</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -2400,7 +2404,7 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>Name of the planning officer who provided the pre-application advice</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2419,7 +2423,7 @@
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Advice date</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -2427,12 +2431,12 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -2446,7 +2450,7 @@
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Advice summary</t>
+          <t>Advice date</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -2454,12 +2458,12 @@
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Summary of the pre-application advice received from the planning authority</t>
+          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -2469,36 +2473,24 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Site details</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Where the proposed development will be built.</t>
-        </is>
-      </c>
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Site boundary</t>
-        </is>
-      </c>
+          <t>Advice summary</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Geometry of the site of the development, typically in GeoJSON format</t>
+          <t>Summary of the pre-application advice received from the planning authority</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>wkt</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -2508,8 +2500,16 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Site details</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Where the proposed development will be built.</t>
+        </is>
+      </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Site locations[]</t>
@@ -2517,19 +2517,19 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Site boundary</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>Geometry of the site of the development, typically in GeoJSON format</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>wkt</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -2548,14 +2548,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -2579,19 +2579,19 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Easting</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -2610,19 +2610,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Northing</t>
+          <t>Easting</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
+          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -2641,19 +2641,19 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Northing</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -2672,19 +2672,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -2703,19 +2703,19 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>A text description providing details about the subject. For parking changes, this describes how the proposed works affect existing car parking arrangements.</t>
+          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -2734,14 +2734,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>UPRNs[]</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
+          <t>A text description providing details about the subject.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -2756,46 +2756,50 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Site Visit Details</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Information to help the planning authority arrange a site visit</t>
-        </is>
-      </c>
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Site seen from public area</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr"/>
+          <t>Site locations[]</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>UPRNs[]</t>
+        </is>
+      </c>
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
+          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
-      <c r="B72" s="2" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Site Visit Details</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Information to help the planning authority arrange a site visit</t>
+        </is>
+      </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Site visit contact type</t>
+          <t>Site seen from public area</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
@@ -2803,12 +2807,12 @@
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Indicates who the authority should contact to arrange a site visit</t>
+          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -2822,7 +2826,7 @@
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Contact reference</t>
+          <t>Site visit contact type</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
@@ -2830,17 +2834,17 @@
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>The reference of the applicant or agent who should be contacted for site visits</t>
+          <t>Indicates who the authority should contact to arrange a site visit</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2849,19 +2853,15 @@
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Full name</t>
-        </is>
-      </c>
+          <t>Contact reference</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>The complete name of a person</t>
+          <t>The reference of the applicant or agent who should be contacted for site visits</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2885,14 +2885,14 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The complete name of a person</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -2916,22 +2916,53 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
+          <t>A phone number</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
           <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
@@ -2939,34 +2970,34 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B35:B40"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="A57:A61"/>
-    <mergeCell ref="B41"/>
-    <mergeCell ref="B2:B18"/>
-    <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A43:A45"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="B54"/>
-    <mergeCell ref="B46:B53"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="A62:A70"/>
-    <mergeCell ref="B23:B30"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="A2:A18"/>
-    <mergeCell ref="A54"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="A46:A53"/>
+    <mergeCell ref="B55"/>
+    <mergeCell ref="A43"/>
+    <mergeCell ref="A2:A19"/>
+    <mergeCell ref="A24:A31"/>
+    <mergeCell ref="B47:B54"/>
+    <mergeCell ref="B72:B77"/>
+    <mergeCell ref="A36:A41"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="A63:A71"/>
+    <mergeCell ref="A58:A62"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B43"/>
+    <mergeCell ref="A20:A23"/>
     <mergeCell ref="B42"/>
-    <mergeCell ref="A41"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="B62:B70"/>
-    <mergeCell ref="A35:A40"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="B57:B61"/>
-    <mergeCell ref="A23:A30"/>
+    <mergeCell ref="B63:B71"/>
+    <mergeCell ref="B58:B62"/>
+    <mergeCell ref="B36:B41"/>
+    <mergeCell ref="A55"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="A47:A54"/>
+    <mergeCell ref="A72:A77"/>
+    <mergeCell ref="B2:B19"/>
+    <mergeCell ref="B24:B31"/>
     <mergeCell ref="A42"/>
+    <mergeCell ref="B32:B35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>